<commit_message>
feat: Add worker meal cost field and responsive UI adjustments
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -21,12 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -56,10 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23808,7 +23801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23927,53 +23920,6 @@
           <t>수량</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B2" t="n">
-        <v>409</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>-40</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>가산~가평 현장 사용 (자동 차감)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>부장 주진철, 부장 박광복, 주임 김성렬</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24037,7 +23983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CL2"/>
+  <dimension ref="A1:CL1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24490,236 +24436,6 @@
         <is>
           <t>기술료</t>
         </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n">
-        <v>46200</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>409</v>
-      </c>
-      <c r="D2" t="n">
-        <v>40</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="1" t="n">
-        <v>46200.50579772082</v>
-      </c>
-      <c r="G2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>R-RAY(Se-75)</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>40</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>124865</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>4994591</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~19:00</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~19:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr">
-        <is>
-          <t>주임 김성렬</t>
-        </is>
-      </c>
-      <c r="AC2" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~19:00</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>75,000</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>1</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>가스공사</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>KS B 0845</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>매</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>휴일</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>Ir-192 또는 Se-75 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr">
-        <is>
-          <t>15mm 이하 (1.0)</t>
-        </is>
-      </c>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>40</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>135160</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>2550240</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>2040192</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>268999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix stock recommendation bugs and add delete feature
- AI 추천 매수 종목 목록에 사용자 추가 종목이 중복으로 표시되는 문제 수정
- 코스피(.KS)/코스닥(.KQ) 종목 코드를 잘못 기입했을 때 자동으로 상호 변환하여 데이터를 수집하는 자동 대체 로직 추가
- 사용자 추가 종목과 기본 포트폴리오 종목 중복 생성 방지 및 수량 병합 처리
- '나의 실제 보유 주식 현황' 프레임 하단에 '선택 주식 삭제' 기능(버튼) 추가 및 삭제 연동 구현
- '나의 실제 보유 주식 현황' 내역 더블클릭 시 5일 가격 예측 전망 창 열리도록 바인딩
- AI 보유 주식 정밀 진단 시 실제 컬럼명('보유')과 불일치하여 데이터를 읽지 못하던 버그 수정
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -21,7 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -51,8 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23801,7 +23805,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23920,6 +23924,69 @@
           <t>수량</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B2" t="n">
+        <v>409</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-20</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>가산~가평 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>부장 주진철, 부장 박광복</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>가산~가평</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23983,7 +24050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CL1"/>
+  <dimension ref="A1:CW2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24436,6 +24503,276 @@
         <is>
           <t>기술료</t>
         </is>
+      </c>
+      <c r="CM1" t="inlineStr">
+        <is>
+          <t>Meal</t>
+        </is>
+      </c>
+      <c r="CN1" t="inlineStr">
+        <is>
+          <t>Meal2</t>
+        </is>
+      </c>
+      <c r="CO1" t="inlineStr">
+        <is>
+          <t>Meal3</t>
+        </is>
+      </c>
+      <c r="CP1" t="inlineStr">
+        <is>
+          <t>Meal4</t>
+        </is>
+      </c>
+      <c r="CQ1" t="inlineStr">
+        <is>
+          <t>Meal5</t>
+        </is>
+      </c>
+      <c r="CR1" t="inlineStr">
+        <is>
+          <t>Meal6</t>
+        </is>
+      </c>
+      <c r="CS1" t="inlineStr">
+        <is>
+          <t>Meal7</t>
+        </is>
+      </c>
+      <c r="CT1" t="inlineStr">
+        <is>
+          <t>Meal8</t>
+        </is>
+      </c>
+      <c r="CU1" t="inlineStr">
+        <is>
+          <t>Meal9</t>
+        </is>
+      </c>
+      <c r="CV1" t="inlineStr">
+        <is>
+          <t>Meal10</t>
+        </is>
+      </c>
+      <c r="CW1" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>가산~가평</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>409</v>
+      </c>
+      <c r="D2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="1" t="n">
+        <v>46205.35210626158</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Se-75</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>129198</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2583952</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr"/>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr"/>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>가스공사</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr"/>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>Ir-192 또는 Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>15mm 초과 ~ 25mm 이하 (1.4)</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>28</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>177340</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>1262996</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>1010396</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>133220</v>
+      </c>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix UI layouts and delete entry regex bug
- Fixed bug where deleting recent entry crashed if site name had parentheses by adding regex=False to str.contains
- Adjusted right panel width in Billing Contract Management tab to 1/3 (2:1 ratio)
- Fixed NDT detail frame layout by breaking long rows into multiple rows to prevent horizontal expansion
- Enforced minsize=550 for worker records panel so '일비' column is always visible
- Added functionality to save and restore column widths for tv_recent
- Added '구분' (Location Type) column to tv_recent in Daily Work Report tab
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -21,10 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -54,9 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23805,7 +23801,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23924,69 +23920,6 @@
           <t>수량</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B2" t="n">
-        <v>409</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>-35</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>가산~가평 현장 사용 (자동 차감)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>부장 주진철, 대리 우명광</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24050,7 +23983,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DA2"/>
+  <dimension ref="A1:DA1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24576,247 +24509,8 @@
       </c>
       <c r="DA1" t="inlineStr">
         <is>
-          <t>수량</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46224</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>409</v>
-      </c>
-      <c r="D2" t="n">
-        <v>35</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="1" t="n">
-        <v>46224.76518125</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>Se-75</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>35</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>94817</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>3318612</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>RT</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>대리 우명광</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>한국가스공사</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr"/>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>매</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>Ir-192 또는 Se-75 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr">
-        <is>
-          <t>15mm 이하 (1.0)</t>
-        </is>
-      </c>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>35</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>310345</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>1578745</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>1262996</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>166526</v>
-      </c>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
-      <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr"/>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr"/>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX2" t="n">
-        <v>7</v>
-      </c>
-      <c r="CY2" t="inlineStr"/>
-      <c r="CZ2" t="n">
-        <v>20</v>
-      </c>
-      <c r="DA2" t="n">
-        <v>0</v>
+          <t>구분</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add and improve PDF Editor script (pdf편잡_editor.py)
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -51,8 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -23801,7 +23808,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23920,6 +23927,53 @@
           <t>수량</t>
         </is>
       </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B2" t="n">
+        <v>406</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>OUT</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>-15</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>가산~가평 현장 사용 (자동 차감)</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>부장 주진철, 대리 우명광</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>가산~가평</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+      <c r="S2" t="inlineStr"/>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23983,7 +24037,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DA1"/>
+  <dimension ref="A1:DA2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24510,6 +24564,255 @@
       <c r="DA1" t="inlineStr">
         <is>
           <t>구분</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n">
+        <v>46226</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>가산~가평</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>406</v>
+      </c>
+      <c r="D2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="1" t="n">
+        <v>46226.34529921455</v>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>Se-75</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>15</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>93975</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>1409632</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>RT</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~21:00</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>대리 우명광</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~21:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="inlineStr"/>
+      <c r="BH2" t="inlineStr"/>
+      <c r="BI2" t="inlineStr"/>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>한국가스공사</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>PIPE</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr"/>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>Ir-192 또는 Se-75 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr">
+        <is>
+          <t>15mm 이하 (1.0)</t>
+        </is>
+      </c>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>15</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>120375</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>676605</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>541284</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>71368</v>
+      </c>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="CY2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="DA2" t="inlineStr">
+        <is>
+          <t>수송배관(주배관)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix memo saving/loading, rename main script, and update default export filename
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S455"/>
+  <dimension ref="A1:S473"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21424,7 +21424,7 @@
         <v>10</v>
       </c>
       <c r="S406" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="407">
@@ -21567,7 +21567,7 @@
         <v>10</v>
       </c>
       <c r="S409" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="410">
@@ -21612,7 +21612,7 @@
         <v>10</v>
       </c>
       <c r="S410" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="411">
@@ -21890,7 +21890,7 @@
         <v>10</v>
       </c>
       <c r="S416" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="417">
@@ -21939,7 +21939,7 @@
         <v>10</v>
       </c>
       <c r="S417" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="418">
@@ -21988,7 +21988,7 @@
         <v>10</v>
       </c>
       <c r="S418" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="419">
@@ -23526,7 +23526,7 @@
         <v>10</v>
       </c>
       <c r="S450" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="451">
@@ -23792,6 +23792,744 @@
       </c>
       <c r="S455" t="n">
         <v>0</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="n">
+        <v>463</v>
+      </c>
+      <c r="B456" t="inlineStr"/>
+      <c r="C456" t="inlineStr"/>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Carestream AA400-10*12"</t>
+        </is>
+      </c>
+      <c r="E456" t="inlineStr"/>
+      <c r="F456" t="inlineStr"/>
+      <c r="G456" t="inlineStr"/>
+      <c r="H456" t="inlineStr"/>
+      <c r="I456" t="inlineStr"/>
+      <c r="J456" t="inlineStr"/>
+      <c r="K456" t="n">
+        <v>0</v>
+      </c>
+      <c r="L456" t="n">
+        <v>0</v>
+      </c>
+      <c r="M456" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N456" t="inlineStr"/>
+      <c r="O456" t="inlineStr"/>
+      <c r="P456" t="inlineStr"/>
+      <c r="Q456" t="n">
+        <v>0</v>
+      </c>
+      <c r="R456" t="n">
+        <v>0</v>
+      </c>
+      <c r="S456" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="n">
+        <v>464</v>
+      </c>
+      <c r="B457" t="inlineStr"/>
+      <c r="C457" t="inlineStr"/>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Carestream AA400-3⅓*12"</t>
+        </is>
+      </c>
+      <c r="E457" t="inlineStr"/>
+      <c r="F457" t="inlineStr"/>
+      <c r="G457" t="inlineStr"/>
+      <c r="H457" t="inlineStr"/>
+      <c r="I457" t="inlineStr"/>
+      <c r="J457" t="inlineStr"/>
+      <c r="K457" t="n">
+        <v>0</v>
+      </c>
+      <c r="L457" t="n">
+        <v>0</v>
+      </c>
+      <c r="M457" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N457" t="inlineStr"/>
+      <c r="O457" t="inlineStr"/>
+      <c r="P457" t="inlineStr"/>
+      <c r="Q457" t="n">
+        <v>0</v>
+      </c>
+      <c r="R457" t="n">
+        <v>0</v>
+      </c>
+      <c r="S457" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="n">
+        <v>465</v>
+      </c>
+      <c r="B458" t="inlineStr"/>
+      <c r="C458" t="inlineStr"/>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Carestream AA400-3⅓*17"</t>
+        </is>
+      </c>
+      <c r="E458" t="inlineStr"/>
+      <c r="F458" t="inlineStr"/>
+      <c r="G458" t="inlineStr"/>
+      <c r="H458" t="inlineStr"/>
+      <c r="I458" t="inlineStr"/>
+      <c r="J458" t="inlineStr"/>
+      <c r="K458" t="n">
+        <v>0</v>
+      </c>
+      <c r="L458" t="n">
+        <v>0</v>
+      </c>
+      <c r="M458" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N458" t="inlineStr"/>
+      <c r="O458" t="inlineStr"/>
+      <c r="P458" t="inlineStr"/>
+      <c r="Q458" t="n">
+        <v>0</v>
+      </c>
+      <c r="R458" t="n">
+        <v>0</v>
+      </c>
+      <c r="S458" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="n">
+        <v>466</v>
+      </c>
+      <c r="B459" t="inlineStr"/>
+      <c r="C459" t="inlineStr"/>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Carestream AA400-4½*12"</t>
+        </is>
+      </c>
+      <c r="E459" t="inlineStr"/>
+      <c r="F459" t="inlineStr"/>
+      <c r="G459" t="inlineStr"/>
+      <c r="H459" t="inlineStr"/>
+      <c r="I459" t="inlineStr"/>
+      <c r="J459" t="inlineStr"/>
+      <c r="K459" t="n">
+        <v>0</v>
+      </c>
+      <c r="L459" t="n">
+        <v>0</v>
+      </c>
+      <c r="M459" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N459" t="inlineStr"/>
+      <c r="O459" t="inlineStr"/>
+      <c r="P459" t="inlineStr"/>
+      <c r="Q459" t="n">
+        <v>0</v>
+      </c>
+      <c r="R459" t="n">
+        <v>0</v>
+      </c>
+      <c r="S459" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="n">
+        <v>467</v>
+      </c>
+      <c r="B460" t="inlineStr"/>
+      <c r="C460" t="inlineStr"/>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Carestream M100-10*12"</t>
+        </is>
+      </c>
+      <c r="E460" t="inlineStr"/>
+      <c r="F460" t="inlineStr"/>
+      <c r="G460" t="inlineStr"/>
+      <c r="H460" t="inlineStr"/>
+      <c r="I460" t="inlineStr"/>
+      <c r="J460" t="inlineStr"/>
+      <c r="K460" t="n">
+        <v>0</v>
+      </c>
+      <c r="L460" t="n">
+        <v>0</v>
+      </c>
+      <c r="M460" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N460" t="inlineStr"/>
+      <c r="O460" t="inlineStr"/>
+      <c r="P460" t="inlineStr"/>
+      <c r="Q460" t="n">
+        <v>0</v>
+      </c>
+      <c r="R460" t="n">
+        <v>0</v>
+      </c>
+      <c r="S460" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="n">
+        <v>468</v>
+      </c>
+      <c r="B461" t="inlineStr"/>
+      <c r="C461" t="inlineStr"/>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Carestream M100-14*17"</t>
+        </is>
+      </c>
+      <c r="E461" t="inlineStr"/>
+      <c r="F461" t="inlineStr"/>
+      <c r="G461" t="inlineStr"/>
+      <c r="H461" t="inlineStr"/>
+      <c r="I461" t="inlineStr"/>
+      <c r="J461" t="inlineStr"/>
+      <c r="K461" t="n">
+        <v>0</v>
+      </c>
+      <c r="L461" t="n">
+        <v>0</v>
+      </c>
+      <c r="M461" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N461" t="inlineStr"/>
+      <c r="O461" t="inlineStr"/>
+      <c r="P461" t="inlineStr"/>
+      <c r="Q461" t="n">
+        <v>0</v>
+      </c>
+      <c r="R461" t="n">
+        <v>0</v>
+      </c>
+      <c r="S461" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="n">
+        <v>469</v>
+      </c>
+      <c r="B462" t="inlineStr"/>
+      <c r="C462" t="inlineStr"/>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Carestream M100-3⅓*12"</t>
+        </is>
+      </c>
+      <c r="E462" t="inlineStr"/>
+      <c r="F462" t="inlineStr"/>
+      <c r="G462" t="inlineStr"/>
+      <c r="H462" t="inlineStr"/>
+      <c r="I462" t="inlineStr"/>
+      <c r="J462" t="inlineStr"/>
+      <c r="K462" t="n">
+        <v>0</v>
+      </c>
+      <c r="L462" t="n">
+        <v>0</v>
+      </c>
+      <c r="M462" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N462" t="inlineStr"/>
+      <c r="O462" t="inlineStr"/>
+      <c r="P462" t="inlineStr"/>
+      <c r="Q462" t="n">
+        <v>0</v>
+      </c>
+      <c r="R462" t="n">
+        <v>0</v>
+      </c>
+      <c r="S462" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="n">
+        <v>470</v>
+      </c>
+      <c r="B463" t="inlineStr"/>
+      <c r="C463" t="inlineStr"/>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Carestream MX125-10*12"</t>
+        </is>
+      </c>
+      <c r="E463" t="inlineStr"/>
+      <c r="F463" t="inlineStr"/>
+      <c r="G463" t="inlineStr"/>
+      <c r="H463" t="inlineStr"/>
+      <c r="I463" t="inlineStr"/>
+      <c r="J463" t="inlineStr"/>
+      <c r="K463" t="n">
+        <v>0</v>
+      </c>
+      <c r="L463" t="n">
+        <v>0</v>
+      </c>
+      <c r="M463" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N463" t="inlineStr"/>
+      <c r="O463" t="inlineStr"/>
+      <c r="P463" t="inlineStr"/>
+      <c r="Q463" t="n">
+        <v>0</v>
+      </c>
+      <c r="R463" t="n">
+        <v>0</v>
+      </c>
+      <c r="S463" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="n">
+        <v>471</v>
+      </c>
+      <c r="B464" t="inlineStr"/>
+      <c r="C464" t="inlineStr"/>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Carestream MX125-14*17"</t>
+        </is>
+      </c>
+      <c r="E464" t="inlineStr"/>
+      <c r="F464" t="inlineStr"/>
+      <c r="G464" t="inlineStr"/>
+      <c r="H464" t="inlineStr"/>
+      <c r="I464" t="inlineStr"/>
+      <c r="J464" t="inlineStr"/>
+      <c r="K464" t="n">
+        <v>0</v>
+      </c>
+      <c r="L464" t="n">
+        <v>0</v>
+      </c>
+      <c r="M464" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N464" t="inlineStr"/>
+      <c r="O464" t="inlineStr"/>
+      <c r="P464" t="inlineStr"/>
+      <c r="Q464" t="n">
+        <v>0</v>
+      </c>
+      <c r="R464" t="n">
+        <v>0</v>
+      </c>
+      <c r="S464" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="n">
+        <v>472</v>
+      </c>
+      <c r="B465" t="inlineStr"/>
+      <c r="C465" t="inlineStr"/>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Carestream MX125-3⅓*12"</t>
+        </is>
+      </c>
+      <c r="E465" t="inlineStr"/>
+      <c r="F465" t="inlineStr"/>
+      <c r="G465" t="inlineStr"/>
+      <c r="H465" t="inlineStr"/>
+      <c r="I465" t="inlineStr"/>
+      <c r="J465" t="inlineStr"/>
+      <c r="K465" t="n">
+        <v>0</v>
+      </c>
+      <c r="L465" t="n">
+        <v>0</v>
+      </c>
+      <c r="M465" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N465" t="inlineStr"/>
+      <c r="O465" t="inlineStr"/>
+      <c r="P465" t="inlineStr"/>
+      <c r="Q465" t="n">
+        <v>0</v>
+      </c>
+      <c r="R465" t="n">
+        <v>0</v>
+      </c>
+      <c r="S465" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="n">
+        <v>473</v>
+      </c>
+      <c r="B466" t="inlineStr"/>
+      <c r="C466" t="inlineStr"/>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Carestream MX125-3⅓*6"</t>
+        </is>
+      </c>
+      <c r="E466" t="inlineStr"/>
+      <c r="F466" t="inlineStr"/>
+      <c r="G466" t="inlineStr"/>
+      <c r="H466" t="inlineStr"/>
+      <c r="I466" t="inlineStr"/>
+      <c r="J466" t="inlineStr"/>
+      <c r="K466" t="n">
+        <v>0</v>
+      </c>
+      <c r="L466" t="n">
+        <v>0</v>
+      </c>
+      <c r="M466" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N466" t="inlineStr"/>
+      <c r="O466" t="inlineStr"/>
+      <c r="P466" t="inlineStr"/>
+      <c r="Q466" t="n">
+        <v>0</v>
+      </c>
+      <c r="R466" t="n">
+        <v>0</v>
+      </c>
+      <c r="S466" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="n">
+        <v>474</v>
+      </c>
+      <c r="B467" t="inlineStr"/>
+      <c r="C467" t="inlineStr"/>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Carestream MX125-4½*12"</t>
+        </is>
+      </c>
+      <c r="E467" t="inlineStr"/>
+      <c r="F467" t="inlineStr"/>
+      <c r="G467" t="inlineStr"/>
+      <c r="H467" t="inlineStr"/>
+      <c r="I467" t="inlineStr"/>
+      <c r="J467" t="inlineStr"/>
+      <c r="K467" t="n">
+        <v>0</v>
+      </c>
+      <c r="L467" t="n">
+        <v>0</v>
+      </c>
+      <c r="M467" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N467" t="inlineStr"/>
+      <c r="O467" t="inlineStr"/>
+      <c r="P467" t="inlineStr"/>
+      <c r="Q467" t="n">
+        <v>0</v>
+      </c>
+      <c r="R467" t="n">
+        <v>0</v>
+      </c>
+      <c r="S467" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="n">
+        <v>475</v>
+      </c>
+      <c r="B468" t="inlineStr"/>
+      <c r="C468" t="inlineStr"/>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Carestream T200-10*12"</t>
+        </is>
+      </c>
+      <c r="E468" t="inlineStr"/>
+      <c r="F468" t="inlineStr"/>
+      <c r="G468" t="inlineStr"/>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr"/>
+      <c r="J468" t="inlineStr"/>
+      <c r="K468" t="n">
+        <v>0</v>
+      </c>
+      <c r="L468" t="n">
+        <v>0</v>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr"/>
+      <c r="O468" t="inlineStr"/>
+      <c r="P468" t="inlineStr"/>
+      <c r="Q468" t="n">
+        <v>0</v>
+      </c>
+      <c r="R468" t="n">
+        <v>0</v>
+      </c>
+      <c r="S468" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="n">
+        <v>476</v>
+      </c>
+      <c r="B469" t="inlineStr"/>
+      <c r="C469" t="inlineStr"/>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Carestream T200-14*17"</t>
+        </is>
+      </c>
+      <c r="E469" t="inlineStr"/>
+      <c r="F469" t="inlineStr"/>
+      <c r="G469" t="inlineStr"/>
+      <c r="H469" t="inlineStr"/>
+      <c r="I469" t="inlineStr"/>
+      <c r="J469" t="inlineStr"/>
+      <c r="K469" t="n">
+        <v>0</v>
+      </c>
+      <c r="L469" t="n">
+        <v>0</v>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr"/>
+      <c r="O469" t="inlineStr"/>
+      <c r="P469" t="inlineStr"/>
+      <c r="Q469" t="n">
+        <v>0</v>
+      </c>
+      <c r="R469" t="n">
+        <v>0</v>
+      </c>
+      <c r="S469" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="n">
+        <v>477</v>
+      </c>
+      <c r="B470" t="inlineStr"/>
+      <c r="C470" t="inlineStr"/>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Carestream T200-3⅓*12"</t>
+        </is>
+      </c>
+      <c r="E470" t="inlineStr"/>
+      <c r="F470" t="inlineStr"/>
+      <c r="G470" t="inlineStr"/>
+      <c r="H470" t="inlineStr"/>
+      <c r="I470" t="inlineStr"/>
+      <c r="J470" t="inlineStr"/>
+      <c r="K470" t="n">
+        <v>0</v>
+      </c>
+      <c r="L470" t="n">
+        <v>0</v>
+      </c>
+      <c r="M470" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N470" t="inlineStr"/>
+      <c r="O470" t="inlineStr"/>
+      <c r="P470" t="inlineStr"/>
+      <c r="Q470" t="n">
+        <v>0</v>
+      </c>
+      <c r="R470" t="n">
+        <v>0</v>
+      </c>
+      <c r="S470" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="n">
+        <v>478</v>
+      </c>
+      <c r="B471" t="inlineStr"/>
+      <c r="C471" t="inlineStr"/>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Carestream T200-3⅓*17"</t>
+        </is>
+      </c>
+      <c r="E471" t="inlineStr"/>
+      <c r="F471" t="inlineStr"/>
+      <c r="G471" t="inlineStr"/>
+      <c r="H471" t="inlineStr"/>
+      <c r="I471" t="inlineStr"/>
+      <c r="J471" t="inlineStr"/>
+      <c r="K471" t="n">
+        <v>0</v>
+      </c>
+      <c r="L471" t="n">
+        <v>0</v>
+      </c>
+      <c r="M471" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N471" t="inlineStr"/>
+      <c r="O471" t="inlineStr"/>
+      <c r="P471" t="inlineStr"/>
+      <c r="Q471" t="n">
+        <v>0</v>
+      </c>
+      <c r="R471" t="n">
+        <v>0</v>
+      </c>
+      <c r="S471" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="n">
+        <v>479</v>
+      </c>
+      <c r="B472" t="inlineStr"/>
+      <c r="C472" t="inlineStr"/>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Carestream T200-4½*12"</t>
+        </is>
+      </c>
+      <c r="E472" t="inlineStr"/>
+      <c r="F472" t="inlineStr"/>
+      <c r="G472" t="inlineStr"/>
+      <c r="H472" t="inlineStr"/>
+      <c r="I472" t="inlineStr"/>
+      <c r="J472" t="inlineStr"/>
+      <c r="K472" t="n">
+        <v>0</v>
+      </c>
+      <c r="L472" t="n">
+        <v>0</v>
+      </c>
+      <c r="M472" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N472" t="inlineStr"/>
+      <c r="O472" t="inlineStr"/>
+      <c r="P472" t="inlineStr"/>
+      <c r="Q472" t="n">
+        <v>0</v>
+      </c>
+      <c r="R472" t="n">
+        <v>0</v>
+      </c>
+      <c r="S472" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="n">
+        <v>480</v>
+      </c>
+      <c r="B473" t="inlineStr"/>
+      <c r="C473" t="inlineStr"/>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>JIREH Scanner</t>
+        </is>
+      </c>
+      <c r="E473" t="inlineStr"/>
+      <c r="F473" t="inlineStr"/>
+      <c r="G473" t="inlineStr"/>
+      <c r="H473" t="inlineStr"/>
+      <c r="I473" t="inlineStr"/>
+      <c r="J473" t="inlineStr"/>
+      <c r="K473" t="n">
+        <v>0</v>
+      </c>
+      <c r="L473" t="n">
+        <v>0</v>
+      </c>
+      <c r="M473" t="inlineStr">
+        <is>
+          <t>매</t>
+        </is>
+      </c>
+      <c r="N473" t="inlineStr"/>
+      <c r="O473" t="inlineStr"/>
+      <c r="P473" t="inlineStr"/>
+      <c r="Q473" t="n">
+        <v>0</v>
+      </c>
+      <c r="R473" t="n">
+        <v>0</v>
+      </c>
+      <c r="S473" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -23805,7 +24543,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -23924,69 +24662,6 @@
           <t>수량</t>
         </is>
       </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46226</v>
-      </c>
-      <c r="B2" t="n">
-        <v>406</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>-15</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>가산~가평 현장 사용 (자동 차감)</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>부장 주진철, 대리 우명광</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>가산~가평</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>nan</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
-      <c r="N2" t="inlineStr"/>
-      <c r="O2" t="inlineStr"/>
-      <c r="P2" t="inlineStr"/>
-      <c r="Q2" t="inlineStr"/>
-      <c r="R2" t="inlineStr"/>
-      <c r="S2" t="inlineStr"/>
-      <c r="T2" t="inlineStr"/>
-      <c r="U2" t="inlineStr"/>
-      <c r="V2" t="inlineStr"/>
-      <c r="W2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -24050,7 +24725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DB2"/>
+  <dimension ref="A1:DC2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24581,31 +25256,40 @@
       </c>
       <c r="DB1" t="inlineStr">
         <is>
+          <t>Remark</t>
+        </is>
+      </c>
+      <c r="DC1" t="inlineStr">
+        <is>
           <t>수량</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46226</v>
+        <v>46236</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>가산~가평</t>
+          <t>중앙지사</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>406</v>
+        <v>480</v>
       </c>
       <c r="D2" t="n">
-        <v>15</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
+        <v>10</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>kds;ds;d;skds;kds;kds;</t>
+        </is>
+      </c>
       <c r="F2" s="1" t="n">
-        <v>46226.34529921296</v>
+        <v>46236.52771778935</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -24632,14 +25316,14 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Se-75</t>
+          <t>PAUT MX2(OMNI2-103085)</t>
         </is>
       </c>
       <c r="P2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="Q2" t="n">
-        <v>93975</v>
+        <v>284015</v>
       </c>
       <c r="R2" t="n">
         <v>0</v>
@@ -24648,11 +25332,11 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>1409632</v>
+        <v>2840150</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>RT</t>
+          <t>PAUT</t>
         </is>
       </c>
       <c r="V2" t="n">
@@ -24660,53 +25344,65 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
+          <t>(주간) 09:00~23:00</t>
+        </is>
+      </c>
+      <c r="X2" t="n">
+        <v>105000</v>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>대리 우명광</t>
+          <t>주임 김진환</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
+          <t>(주간) 09:00~23:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="n">
+        <v>105000</v>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
+      <c r="AD2" t="n">
+        <v>0</v>
+      </c>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="n">
+        <v>0</v>
+      </c>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
+      <c r="AJ2" t="n">
+        <v>0</v>
+      </c>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
+      <c r="AM2" t="n">
+        <v>0</v>
+      </c>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
+      <c r="AP2" t="n">
+        <v>0</v>
+      </c>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
+      <c r="AS2" t="n">
+        <v>0</v>
+      </c>
       <c r="AT2" t="inlineStr"/>
       <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
+      <c r="AV2" t="n">
+        <v>0</v>
+      </c>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
+      <c r="AY2" t="n">
+        <v>0</v>
+      </c>
       <c r="AZ2" t="n">
         <v>0</v>
       </c>
@@ -24728,18 +25424,34 @@
       <c r="BF2" t="n">
         <v>0</v>
       </c>
-      <c r="BG2" t="inlineStr"/>
-      <c r="BH2" t="inlineStr"/>
-      <c r="BI2" t="inlineStr"/>
-      <c r="BJ2" t="inlineStr"/>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>81도8458 || 81도 5958</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>123654 || 123564</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr">
+        <is>
+          <t>||</t>
+        </is>
+      </c>
       <c r="BK2" t="inlineStr"/>
       <c r="BL2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr">
         <is>
-          <t>한국가스공사</t>
+          <t>한국지역난방공사 중앙지사</t>
         </is>
       </c>
       <c r="BO2" t="inlineStr"/>
@@ -24751,52 +25463,60 @@
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr"/>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
       <c r="BX2" t="inlineStr"/>
       <c r="BY2" t="inlineStr"/>
       <c r="BZ2" t="inlineStr">
         <is>
-          <t>매</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr">
+        <is>
+          <t>JIREH Scanner</t>
+        </is>
+      </c>
       <c r="CB2" t="inlineStr">
         <is>
-          <t>일반</t>
+          <t>야간</t>
         </is>
       </c>
       <c r="CC2" t="inlineStr">
         <is>
-          <t>Ir-192 또는 Se-75 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr">
-        <is>
-          <t>15mm 이하 (1.0)</t>
-        </is>
-      </c>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF2" t="n">
+        <v>0</v>
+      </c>
       <c r="CG2" t="n">
         <v>1</v>
       </c>
       <c r="CH2" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="CI2" t="n">
-        <v>120375</v>
+        <v>375590</v>
       </c>
       <c r="CJ2" t="n">
-        <v>676605</v>
+        <v>978000</v>
       </c>
       <c r="CK2" t="n">
-        <v>541284</v>
+        <v>1075800</v>
       </c>
       <c r="CL2" t="n">
-        <v>71368</v>
+        <v>410760</v>
       </c>
       <c r="CM2" t="inlineStr"/>
       <c r="CN2" t="inlineStr"/>
@@ -24814,20 +25534,27 @@
         </is>
       </c>
       <c r="CX2" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="CY2" t="n">
         <v>0</v>
       </c>
-      <c r="CZ2" t="n">
-        <v>4</v>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>300A</t>
+        </is>
       </c>
       <c r="DA2" t="inlineStr">
         <is>
-          <t>수송배관(주배관)</t>
-        </is>
-      </c>
-      <c r="DB2" t="n">
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB2" t="inlineStr">
+        <is>
+          <t>안녕하세요? 주진철입니다.</t>
+        </is>
+      </c>
+      <c r="DC2" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update material system and configurations
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -21,9 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25261,32 +25264,30 @@
       </c>
       <c r="DC1" t="inlineStr">
         <is>
-          <t>수량</t>
+          <t>DailyMemo</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46236</v>
+        <v>46237</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
           <t>중앙지사</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>480</v>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>JIREH MICROBE</t>
+        </is>
       </c>
       <c r="D2" t="n">
-        <v>10</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>kds;ds;d;skds;kds;kds;</t>
-        </is>
-      </c>
-      <c r="F2" s="1" t="n">
-        <v>46236.52771778935</v>
+        <v>19.151</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="2" t="n">
+        <v>46237.74883386539</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -25311,7 +25312,7 @@
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>부장 주진철</t>
+          <t>대리 우명광</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -25320,7 +25321,7 @@
         </is>
       </c>
       <c r="P2" t="n">
-        <v>10</v>
+        <v>19.151</v>
       </c>
       <c r="Q2" t="n">
         <v>284015</v>
@@ -25332,7 +25333,7 @@
         <v>0</v>
       </c>
       <c r="T2" t="n">
-        <v>2840150</v>
+        <v>5439168</v>
       </c>
       <c r="U2" t="inlineStr">
         <is>
@@ -25344,65 +25345,53 @@
       </c>
       <c r="W2" t="inlineStr">
         <is>
-          <t>(주간) 09:00~23:00</t>
-        </is>
-      </c>
-      <c r="X2" t="n">
-        <v>105000</v>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
       </c>
       <c r="Y2" t="inlineStr">
         <is>
-          <t>주임 김진환</t>
+          <t>부장 주진철</t>
         </is>
       </c>
       <c r="Z2" t="inlineStr">
         <is>
-          <t>(주간) 09:00~23:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="n">
-        <v>105000</v>
+          <t>(야간) 22:00~익일03:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>25,000</t>
+        </is>
       </c>
       <c r="AB2" t="inlineStr"/>
       <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AD2" t="inlineStr"/>
       <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AG2" t="inlineStr"/>
       <c r="AH2" t="inlineStr"/>
       <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AJ2" t="inlineStr"/>
       <c r="AK2" t="inlineStr"/>
       <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AM2" t="inlineStr"/>
       <c r="AN2" t="inlineStr"/>
       <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="inlineStr"/>
       <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AS2" t="inlineStr"/>
       <c r="AT2" t="inlineStr"/>
       <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AV2" t="inlineStr"/>
       <c r="AW2" t="inlineStr"/>
       <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="n">
-        <v>0</v>
-      </c>
+      <c r="AY2" t="inlineStr"/>
       <c r="AZ2" t="n">
         <v>0</v>
       </c>
@@ -25426,12 +25415,12 @@
       </c>
       <c r="BG2" t="inlineStr">
         <is>
-          <t>81도8458 || 81도 5958</t>
+          <t>81루5100 || 81도5958</t>
         </is>
       </c>
       <c r="BH2" t="inlineStr">
         <is>
-          <t>123654 || 123564</t>
+          <t>123645 || 123654</t>
         </is>
       </c>
       <c r="BI2" t="inlineStr">
@@ -25441,7 +25430,7 @@
       </c>
       <c r="BJ2" t="inlineStr">
         <is>
-          <t>||</t>
+          <t xml:space="preserve"> || </t>
         </is>
       </c>
       <c r="BK2" t="inlineStr"/>
@@ -25451,7 +25440,7 @@
       <c r="BM2" t="inlineStr"/>
       <c r="BN2" t="inlineStr">
         <is>
-          <t>한국지역난방공사 중앙지사</t>
+          <t>한국지역난방공사</t>
         </is>
       </c>
       <c r="BO2" t="inlineStr"/>
@@ -25463,12 +25452,12 @@
       <c r="BU2" t="inlineStr"/>
       <c r="BV2" t="inlineStr">
         <is>
-          <t>Pipe</t>
+          <t>PIPE</t>
         </is>
       </c>
       <c r="BW2" t="inlineStr">
         <is>
-          <t>KS B ISO 13588</t>
+          <t>KS B ISO 13588:2019</t>
         </is>
       </c>
       <c r="BX2" t="inlineStr"/>
@@ -25478,11 +25467,7 @@
           <t>M</t>
         </is>
       </c>
-      <c r="CA2" t="inlineStr">
-        <is>
-          <t>JIREH Scanner</t>
-        </is>
-      </c>
+      <c r="CA2" t="inlineStr"/>
       <c r="CB2" t="inlineStr">
         <is>
           <t>야간</t>
@@ -25494,29 +25479,25 @@
         </is>
       </c>
       <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CF2" t="n">
-        <v>0</v>
-      </c>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
       <c r="CG2" t="n">
         <v>1</v>
       </c>
       <c r="CH2" t="n">
-        <v>10</v>
+        <v>19.151</v>
       </c>
       <c r="CI2" t="n">
-        <v>375590</v>
+        <v>719292</v>
       </c>
       <c r="CJ2" t="n">
-        <v>978000</v>
+        <v>1872967</v>
       </c>
       <c r="CK2" t="n">
-        <v>1075800</v>
+        <v>2060263</v>
       </c>
       <c r="CL2" t="n">
-        <v>410760</v>
+        <v>786646</v>
       </c>
       <c r="CM2" t="inlineStr"/>
       <c r="CN2" t="inlineStr"/>
@@ -25533,15 +25514,19 @@
           <t>ORI</t>
         </is>
       </c>
-      <c r="CX2" t="n">
-        <v>10</v>
-      </c>
-      <c r="CY2" t="n">
-        <v>0</v>
+      <c r="CX2" t="inlineStr">
+        <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="CY2" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="CZ2" t="inlineStr">
         <is>
-          <t>300A</t>
+          <t>600A</t>
         </is>
       </c>
       <c r="DA2" t="inlineStr">
@@ -25549,14 +25534,8 @@
           <t>열배관</t>
         </is>
       </c>
-      <c r="DB2" t="inlineStr">
-        <is>
-          <t>안녕하세요? 주진철입니다.</t>
-        </is>
-      </c>
-      <c r="DC2" t="n">
-        <v>0</v>
-      </c>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update NDT daily log UI: auto-fill quantities, add smart joint auto-increment, and fix global MouseWheel overscroll bug
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -21,11 +21,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -56,10 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24728,7 +24725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DC2"/>
+  <dimension ref="A1:DD2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25267,6 +25264,11 @@
           <t>DailyMemo</t>
         </is>
       </c>
+      <c r="DD1" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
@@ -25277,17 +25279,13 @@
           <t>중앙지사</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>JIREH MICROBE</t>
-        </is>
-      </c>
+      <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>19.151</v>
       </c>
       <c r="E2" t="inlineStr"/>
-      <c r="F2" s="2" t="n">
-        <v>46237.74883386539</v>
+      <c r="F2" s="1" t="n">
+        <v>46237.74883386574</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -25430,7 +25428,7 @@
       </c>
       <c r="BJ2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> || </t>
+          <t>||</t>
         </is>
       </c>
       <c r="BK2" t="inlineStr"/>
@@ -25514,15 +25512,11 @@
           <t>ORI</t>
         </is>
       </c>
-      <c r="CX2" t="inlineStr">
-        <is>
-          <t>10</t>
-        </is>
-      </c>
-      <c r="CY2" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
+      <c r="CX2" t="n">
+        <v>10</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>0</v>
       </c>
       <c r="CZ2" t="inlineStr">
         <is>
@@ -25536,6 +25530,9 @@
       </c>
       <c r="DB2" t="inlineStr"/>
       <c r="DC2" t="inlineStr"/>
+      <c r="DD2" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat: update monthly report workflow and related data
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: improve daily log and progress report handling
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -21,10 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -54,9 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24725,7 +24721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DD2"/>
+  <dimension ref="A1:DC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25263,275 +25259,6 @@
         <is>
           <t>DailyMemo</t>
         </is>
-      </c>
-      <c r="DD1" t="inlineStr">
-        <is>
-          <t>수량</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46237</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="n">
-        <v>19.151</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="1" t="n">
-        <v>46237.74883386574</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>대리 우명광</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>19.151</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>284015</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>5439168</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>(야간) 22:00~익일03:00</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>25,000</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>(야간) 22:00~익일03:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>25,000</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>81루5100 || 81도5958</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>123645 || 123654</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr">
-        <is>
-          <t>||</t>
-        </is>
-      </c>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>한국지역난방공사</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>PIPE</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>KS B ISO 13588:2019</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>야간</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>19.151</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>719292</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>1872967</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>2060263</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>786646</v>
-      </c>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
-      <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr"/>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr"/>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX2" t="n">
-        <v>10</v>
-      </c>
-      <c r="CY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ2" t="inlineStr">
-        <is>
-          <t>600A</t>
-        </is>
-      </c>
-      <c r="DA2" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB2" t="inlineStr"/>
-      <c r="DC2" t="inlineStr"/>
-      <c r="DD2" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fix combobox dropdown behavior, depreciation qty, and update headers
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -51,8 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24721,7 +24725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DC1"/>
+  <dimension ref="A1:DD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25259,6 +25263,797 @@
         <is>
           <t>DailyMemo</t>
         </is>
+      </c>
+      <c r="DD1" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>480</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="1" t="n">
+        <v>46257.92779054398</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>201863</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2061744</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>(휴일) 10:00~17:00</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>52,500</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>(휴일) 10:00~17:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>52,500</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>81도8458 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>383612</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>665926</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>732518</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>279688</v>
+      </c>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX2" t="n">
+        <v>8</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>400A</t>
+        </is>
+      </c>
+      <c r="DA2" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
+      <c r="DD2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>480</v>
+      </c>
+      <c r="D3" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="1" t="n">
+        <v>46257.92952744213</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~21:00</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~21:00</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>81도8458 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr"/>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC3" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>383612</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>665926</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>732518</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>279688</v>
+      </c>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
+      <c r="CQ3" t="inlineStr"/>
+      <c r="CR3" t="inlineStr"/>
+      <c r="CS3" t="inlineStr"/>
+      <c r="CT3" t="inlineStr"/>
+      <c r="CU3" t="inlineStr"/>
+      <c r="CV3" t="inlineStr"/>
+      <c r="CW3" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX3" t="n">
+        <v>8</v>
+      </c>
+      <c r="CY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ3" t="inlineStr">
+        <is>
+          <t>400A</t>
+        </is>
+      </c>
+      <c r="DA3" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB3" t="inlineStr"/>
+      <c r="DC3" t="inlineStr"/>
+      <c r="DD3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>480</v>
+      </c>
+      <c r="D4" t="n">
+        <v>4.0024</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="1" t="n">
+        <v>46257.93140291666</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>4.0024</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>201862</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>807934</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스) || 95가0175 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>60 || 60</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr">
+        <is>
+          <t>||</t>
+        </is>
+      </c>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr"/>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC4" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>4.0024</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>150326</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>260956</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>287051</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>109601</v>
+      </c>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
+      <c r="CQ4" t="inlineStr"/>
+      <c r="CR4" t="inlineStr"/>
+      <c r="CS4" t="inlineStr"/>
+      <c r="CT4" t="inlineStr"/>
+      <c r="CU4" t="inlineStr"/>
+      <c r="CV4" t="inlineStr"/>
+      <c r="CW4" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX4" t="n">
+        <v>4</v>
+      </c>
+      <c r="CY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ4" t="inlineStr">
+        <is>
+          <t>300A</t>
+        </is>
+      </c>
+      <c r="DA4" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB4" t="inlineStr"/>
+      <c r="DC4" t="inlineStr"/>
+      <c r="DD4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -25272,7 +26067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25294,6 +26089,194 @@
       <c r="D1" t="inlineStr">
         <is>
           <t>ExpenseDetail</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>LaborCost</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>MaterialCost</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Expense</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>OutsourceCost</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
+          <t>Actual_Revenue</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Actual_UnitPrice</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Actual_LaborCost</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Actual_MaterialCost</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>Actual_Expense</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>Actual_OutsourceCost</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Actual_Profit</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Actual_Note</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Actual_Period</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Actual_LaborDetail</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Actual_MaterialDetail</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Actual_ExpenseDetail</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": "230,208"}, "\ubd80\uc7a5": {"personnel": "2", "period": "80", "unit_price": "230,208"}, "\ucc28\uc7a5": {"personnel": "1", "period": "15", "unit_price": "198,625"}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": "171,542"}, "\ub300\ub9ac": {"personnel": "1", "period": "30", "unit_price": "158,000"}, "\uacc4\uc7a5": {"personnel": "1", "period": "20", "unit_price": "144,458"}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": "130,917"}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": "121,875"}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "5", "period": "80", "unit_price": "4,000"}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "5", "period": "80", "unit_price": "5,000"}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "5", "period": "100", "unit_price": "7,500"}}</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>[{"qty": "6", "price": "1,500"}, {"qty": "3", "price": "2,300"}, {"qty": "6", "price": "2,000"}, {"qty": "6", "price": "2,350"}, {"qty": "6", "price": "1,800"}, {"qty": "490", "price": "990"}, {"qty": "2", "price": "100,000"}, {"qty": "8", "price": "16,500"}, {"qty": "8", "price": "16,500"}, {"qty": "8", "price": "2,500"}]</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "N/A", "qty": "80", "unit": "\uc77c", "price": "5,000", "amount": "400,000"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "80", "unit": "\uc77c", "price": "500", "amount": "40,000"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "80", "unit": "\uc77c", "price": "1,667", "amount": "133,360"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "30", "unit": "\uc77c", "price": "35,714", "amount": "1,071,420"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "80", "rate": "44,444", "amount": "3,555,520"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "80", "rate": "5,556", "amount": "444,480"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "10", "rate": "16,667", "amount": "166,670"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "10", "rate": "222", "amount": "2,220"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "30", "rate": "16,667", "amount": "500,010"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "2", "days": "80", "rate": "16,667", "amount": "2,666,720"}]}</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>288268000</v>
+      </c>
+      <c r="G2" t="n">
+        <v>54791815</v>
+      </c>
+      <c r="H2" t="n">
+        <v>1021900</v>
+      </c>
+      <c r="I2" t="n">
+        <v>14824550</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>217629735</v>
+      </c>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="inlineStr"/>
+      <c r="U2" t="inlineStr"/>
+      <c r="V2" t="inlineStr"/>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>{}</t>
         </is>
       </c>
     </row>
@@ -25817,7 +26800,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>EA</t>
+          <t>일</t>
         </is>
       </c>
       <c r="E23" t="n">

</xml_diff>

<commit_message>
Fix actual cost depreciation quantity logic to prevent double counting
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -26067,7 +26067,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y2"/>
+  <dimension ref="A1:Y3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -26277,6 +26277,107 @@
       <c r="Y2" t="inlineStr">
         <is>
           <t>{}</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>0</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": "230,208"}, "\ubd80\uc7a5": {"personnel": "2", "period": "80", "unit_price": "230,208"}, "\ucc28\uc7a5": {"personnel": "1", "period": "15", "unit_price": "198,625"}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": "171,542"}, "\ub300\ub9ac": {"personnel": "1", "period": "30", "unit_price": "158,000"}, "\uacc4\uc7a5": {"personnel": "1", "period": "20", "unit_price": "144,458"}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": "130,917"}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": "121,875"}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "5", "period": "80", "unit_price": "4,000"}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "5", "period": "80", "unit_price": "5,000"}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "5", "period": "100", "unit_price": "7,500"}}</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[{"qty": "6", "price": "1,500"}, {"qty": "3", "price": "2,300"}, {"qty": "6", "price": "2,000"}, {"qty": "6", "price": "2,350"}, {"qty": "6", "price": "1,800"}, {"qty": "490", "price": "990"}, {"qty": "2", "price": "100,000"}, {"qty": "8", "price": "16,500"}, {"qty": "8", "price": "16,500"}, {"qty": "8", "price": "2,500"}]</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "N/A", "qty": "80", "unit": "\uc77c", "price": "5,000", "amount": "400,000"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "80", "unit": "\uc77c", "price": "500", "amount": "40,000"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "80", "unit": "\uc77c", "price": "1,667", "amount": "133,360"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "30", "unit": "\uc77c", "price": "35,714", "amount": "1,071,420"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "80", "rate": "44,444", "amount": "3,555,520"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "80", "rate": "5,556", "amount": "444,480"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "10", "rate": "16,667", "amount": "166,670"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "10", "rate": "222", "amount": "2,220"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "30", "rate": "16,667", "amount": "500,010"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "2", "days": "80", "rate": "16,667", "amount": "2,666,720"}]}</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>288268000</v>
+      </c>
+      <c r="G3" t="n">
+        <v>54791815</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1021900</v>
+      </c>
+      <c r="I3" t="n">
+        <v>14824550</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>217629735</v>
+      </c>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>4931422.0</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>4931422.0</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>1645248.0</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>413652.0</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>2872522.0</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>2026.08.04~2027.08.05</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>{"\uc774\uc0ac": {"personnel": "", "period": "", "unit_price": "230,208"}, "\ubd80\uc7a5": {"personnel": "2", "period": "3", "unit_price": "230,208"}, "\ucc28\uc7a5": {"personnel": "", "period": "", "unit_price": "198,625"}, "\uacfc\uc7a5": {"personnel": "", "period": "", "unit_price": "171,542"}, "\ub300\ub9ac": {"personnel": "", "period": "", "unit_price": "158,000"}, "\uacc4\uc7a5": {"personnel": "", "period": "", "unit_price": "144,458"}, "\uc8fc\uc784": {"personnel": "", "period": "", "unit_price": "130,917"}, "\uae30\uc0ac": {"personnel": "", "period": "", "unit_price": "121,875"}, "\uc5f0\uc7a5\uadfc\ubb34": {"personnel": "2", "period": "3", "unit_price": "4,000"}, "\uc57c\uac04\uadfc\ubb34": {"personnel": "", "period": "", "unit_price": "5,000"}, "\ud734\uc77c\uadfc\ubb34": {"personnel": "2", "period": "16", "unit_price": "7,500"}}</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>[{"qty": "", "price": "1,500"}, {"qty": "", "price": "2,300"}, {"qty": "", "price": "2,000"}, {"qty": "", "price": "2,350"}, {"qty": "", "price": "1,800"}, {"qty": "", "price": "990"}, {"qty": "", "price": "100,000"}, {"qty": "", "price": "16,500"}, {"qty": "", "price": "16,500"}, {"qty": "", "price": "2,500"}]</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>{"site_expense": [{"cat": "\ucc28\ub7c9\uc720\uc9c0\ube44", "cont": "\uc8fc\uc720, \uc218\ub9ac, \ud1b5\ud589, \uc8fc\ucc28 \ub4f1", "ppl": "N/A", "qty": "4", "unit": "\uc77c", "price": "5,000", "amount": "20,000"}, {"cat": "\uc18c\ubaa8\ud488\ube44", "cont": "\uc7a5\uac11,\uc77c\ud68c\uc6a9 \uc791\uc5c5\ubcf5\uc678", "ppl": "N/A", "qty": "3", "unit": "\uc77c", "price": "500", "amount": "1,500"}, {"cat": "\ubcf5\ub9ac\ud6c4\uc0dd\ube44", "cont": "\uc0dd\uc218, \uc74c\ub8cc \uc678 \uae30\ud0c0", "ppl": "N/A", "qty": "", "unit": "\uc77c", "price": "1,667", "amount": "0"}, {"cat": "Se-175", "cont": "\ubc29\uc0ac\uc131\ub3d9\uc704\uc6d0\uc18c \uad6c\ub9e4", "ppl": "N/A", "qty": "", "unit": "\uc77c", "price": "35,714", "amount": "0"}], "rental": [{"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}, {"cat": "", "spec": "", "qty": "", "period": "", "unit": "", "price": "0", "amount": "0"}], "outsource": [{"cat": "\ucf00\uc774\uc5d4\ub514\uc774", "work": "\ubc29\uc0ac\uc120\ud22c\uacfc\uac80\uc0ac", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}, {"cat": "", "work": "", "count": "0", "price": "0", "amount": "0"}], "depreciation": [{"item": "PAUT \uc7a5\ube44", "spec": "", "life": "5", "qty": "1", "days": "3", "rate": "44,444", "amount": "133,332"}, {"item": "PAUT SCANNER (MANUAL)", "spec": "", "life": "5", "qty": "1", "days": "3", "rate": "5,556", "amount": "16,668"}, {"item": "PAUT SCANNER (COBRA)", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "YOKE", "spec": "", "life": "5", "qty": "1", "days": "", "rate": "222", "amount": "0"}, {"item": "\ud604\uc0c1\uc6a9 \ud0d1\ucc28(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \ud0d1\ucc28 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "", "rate": "16,667", "amount": "0"}, {"item": "\uc2a4\ud0c0\ub809\uc2a4(5\ub144\uac04 \ubcf4\ud5d8\ube44 \ud3ec\ud568)", "spec": "\ud604\uc7a5\ubcc4 \ucc28\ub7c9\uae30\uc785\uc2dc \uc2a4\ud0c0\ub809\uc2a4 \uad6c\ubd84 \uae30\uc785", "life": "5", "qty": "1", "days": "4", "rate": "16,667", "amount": "66,668"}]}</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix daily usage save duplicate bug and transaction rollback bug
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,9 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -54,9 +56,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -25534,7 +25537,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46241</v>
+        <v>46256</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -25545,11 +25548,11 @@
         <v>480</v>
       </c>
       <c r="D3" t="n">
-        <v>10.2136</v>
+        <v>4.0024</v>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" s="1" t="n">
-        <v>46257.92952744213</v>
+        <v>46257.93140291666</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -25583,10 +25586,10 @@
         </is>
       </c>
       <c r="P3" t="n">
-        <v>10.2136</v>
+        <v>4.0024</v>
       </c>
       <c r="Q3" t="n">
-        <v>0</v>
+        <v>201862</v>
       </c>
       <c r="R3" t="n">
         <v>0</v>
@@ -25595,7 +25598,7 @@
         <v>0</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>807934</v>
       </c>
       <c r="U3" t="inlineStr">
         <is>
@@ -25607,12 +25610,12 @@
       </c>
       <c r="W3" t="inlineStr">
         <is>
-          <t>(주간) 09:00~21:00</t>
+          <t>(휴일) 09:00~18:00</t>
         </is>
       </c>
       <c r="X3" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>67,500</t>
         </is>
       </c>
       <c r="Y3" t="inlineStr">
@@ -25622,12 +25625,12 @@
       </c>
       <c r="Z3" t="inlineStr">
         <is>
-          <t>(주간) 09:00~21:00</t>
+          <t>(휴일) 09:00~18:00</t>
         </is>
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>12,000</t>
+          <t>67,500</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr"/>
@@ -25677,20 +25680,24 @@
       </c>
       <c r="BG3" t="inlineStr">
         <is>
-          <t>81도8458 (스타렉스)</t>
+          <t>91주8839 (스타렉스) || 95가0175 (스타렉스)</t>
         </is>
       </c>
       <c r="BH3" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>60 || 60</t>
         </is>
       </c>
       <c r="BI3" t="inlineStr">
         <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ3" t="inlineStr"/>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>||</t>
+        </is>
+      </c>
       <c r="BK3" t="inlineStr"/>
       <c r="BL3" t="n">
         <v>0</v>
@@ -25713,11 +25720,7 @@
           <t>Pipe</t>
         </is>
       </c>
-      <c r="BW3" t="inlineStr">
-        <is>
-          <t>KS B ISO 13588</t>
-        </is>
-      </c>
+      <c r="BW3" t="inlineStr"/>
       <c r="BX3" t="inlineStr"/>
       <c r="BY3" t="inlineStr"/>
       <c r="BZ3" t="inlineStr">
@@ -25743,19 +25746,19 @@
         <v>1</v>
       </c>
       <c r="CH3" t="n">
-        <v>10.2136</v>
+        <v>4.0024</v>
       </c>
       <c r="CI3" t="n">
-        <v>383612</v>
+        <v>150326</v>
       </c>
       <c r="CJ3" t="n">
-        <v>665926</v>
+        <v>260956</v>
       </c>
       <c r="CK3" t="n">
-        <v>732518</v>
+        <v>287051</v>
       </c>
       <c r="CL3" t="n">
-        <v>279688</v>
+        <v>109601</v>
       </c>
       <c r="CM3" t="inlineStr"/>
       <c r="CN3" t="inlineStr"/>
@@ -25773,14 +25776,14 @@
         </is>
       </c>
       <c r="CX3" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="CY3" t="n">
         <v>0</v>
       </c>
       <c r="CZ3" t="inlineStr">
         <is>
-          <t>400A</t>
+          <t>300A</t>
         </is>
       </c>
       <c r="DA3" t="inlineStr">
@@ -25795,8 +25798,8 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46256</v>
+      <c r="A4" s="2" t="n">
+        <v>46241</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
@@ -25807,11 +25810,11 @@
         <v>480</v>
       </c>
       <c r="D4" t="n">
-        <v>4.0024</v>
+        <v>10.2136</v>
       </c>
       <c r="E4" t="inlineStr"/>
       <c r="F4" s="1" t="n">
-        <v>46257.93140291666</v>
+        <v>46258.37184411965</v>
       </c>
       <c r="G4" t="n">
         <v>0</v>
@@ -25845,10 +25848,10 @@
         </is>
       </c>
       <c r="P4" t="n">
-        <v>4.0024</v>
+        <v>10.2136</v>
       </c>
       <c r="Q4" t="n">
-        <v>201862</v>
+        <v>201863</v>
       </c>
       <c r="R4" t="n">
         <v>0</v>
@@ -25857,7 +25860,7 @@
         <v>0</v>
       </c>
       <c r="T4" t="n">
-        <v>807934</v>
+        <v>2061744</v>
       </c>
       <c r="U4" t="inlineStr">
         <is>
@@ -25869,12 +25872,12 @@
       </c>
       <c r="W4" t="inlineStr">
         <is>
-          <t>(휴일) 09:00~18:00</t>
+          <t>(주간) 09:00~21:00</t>
         </is>
       </c>
       <c r="X4" t="inlineStr">
         <is>
-          <t>67,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="Y4" t="inlineStr">
@@ -25884,12 +25887,12 @@
       </c>
       <c r="Z4" t="inlineStr">
         <is>
-          <t>(휴일) 09:00~18:00</t>
+          <t>(주간) 09:00~21:00</t>
         </is>
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t>67,500</t>
+          <t>12,000</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr"/>
@@ -25939,24 +25942,20 @@
       </c>
       <c r="BG4" t="inlineStr">
         <is>
-          <t>91주8839 (스타렉스) || 95가0175 (스타렉스)</t>
+          <t>81도8458 (스타렉스)</t>
         </is>
       </c>
       <c r="BH4" t="inlineStr">
         <is>
-          <t>60 || 60</t>
+          <t>60</t>
         </is>
       </c>
       <c r="BI4" t="inlineStr">
         <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ4" t="inlineStr">
-        <is>
-          <t>||</t>
-        </is>
-      </c>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr"/>
       <c r="BK4" t="inlineStr"/>
       <c r="BL4" t="n">
         <v>0</v>
@@ -25979,7 +25978,11 @@
           <t>Pipe</t>
         </is>
       </c>
-      <c r="BW4" t="inlineStr"/>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
       <c r="BX4" t="inlineStr"/>
       <c r="BY4" t="inlineStr"/>
       <c r="BZ4" t="inlineStr">
@@ -26005,19 +26008,19 @@
         <v>1</v>
       </c>
       <c r="CH4" t="n">
-        <v>4.0024</v>
+        <v>10.2136</v>
       </c>
       <c r="CI4" t="n">
-        <v>150326</v>
+        <v>383612</v>
       </c>
       <c r="CJ4" t="n">
-        <v>260956</v>
+        <v>665926</v>
       </c>
       <c r="CK4" t="n">
-        <v>287051</v>
+        <v>732518</v>
       </c>
       <c r="CL4" t="n">
-        <v>109601</v>
+        <v>279688</v>
       </c>
       <c r="CM4" t="inlineStr"/>
       <c r="CN4" t="inlineStr"/>
@@ -26034,15 +26037,19 @@
           <t>ORI</t>
         </is>
       </c>
-      <c r="CX4" t="n">
-        <v>4</v>
-      </c>
-      <c r="CY4" t="n">
-        <v>0</v>
+      <c r="CX4" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="CY4" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
       </c>
       <c r="CZ4" t="inlineStr">
         <is>
-          <t>300A</t>
+          <t>400A</t>
         </is>
       </c>
       <c r="DA4" t="inlineStr">
@@ -26052,9 +26059,7 @@
       </c>
       <c r="DB4" t="inlineStr"/>
       <c r="DC4" t="inlineStr"/>
-      <c r="DD4" t="n">
-        <v>0</v>
-      </c>
+      <c r="DD4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -26323,40 +26328,26 @@
         <v>217629735</v>
       </c>
       <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>4931422.0</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>4931422.0</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>1645248.0</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>413652.0</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>2872522.0</t>
-        </is>
+      <c r="M3" t="n">
+        <v>4931422</v>
+      </c>
+      <c r="N3" t="n">
+        <v>4931422</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1645248</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>413652</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>2872522</v>
       </c>
       <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">

</xml_diff>

<commit_message>
feat: Add MT report generation tab and template logic
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
feat: Separate KOGAS and Joongang databases and fix daily log bugs
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,7 +21,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -51,8 +54,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24721,7 +24725,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DC1"/>
+  <dimension ref="A1:DD4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25259,6 +25263,797 @@
         <is>
           <t>DailyMemo</t>
         </is>
+      </c>
+      <c r="DD1" t="inlineStr">
+        <is>
+          <t>수량</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>46242</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>480</v>
+      </c>
+      <c r="D2" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" s="1" t="n">
+        <v>46257.92779054398</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>201863</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2061744</v>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>(휴일) 10:00~17:00</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>52,500</t>
+        </is>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>(휴일) 10:00~17:00</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>52,500</t>
+        </is>
+      </c>
+      <c r="AB2" t="inlineStr"/>
+      <c r="AC2" t="inlineStr"/>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
+      <c r="AF2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr"/>
+      <c r="AH2" t="inlineStr"/>
+      <c r="AI2" t="inlineStr"/>
+      <c r="AJ2" t="inlineStr"/>
+      <c r="AK2" t="inlineStr"/>
+      <c r="AL2" t="inlineStr"/>
+      <c r="AM2" t="inlineStr"/>
+      <c r="AN2" t="inlineStr"/>
+      <c r="AO2" t="inlineStr"/>
+      <c r="AP2" t="inlineStr"/>
+      <c r="AQ2" t="inlineStr"/>
+      <c r="AR2" t="inlineStr"/>
+      <c r="AS2" t="inlineStr"/>
+      <c r="AT2" t="inlineStr"/>
+      <c r="AU2" t="inlineStr"/>
+      <c r="AV2" t="inlineStr"/>
+      <c r="AW2" t="inlineStr"/>
+      <c r="AX2" t="inlineStr"/>
+      <c r="AY2" t="inlineStr"/>
+      <c r="AZ2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG2" t="inlineStr">
+        <is>
+          <t>81도8458 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI2" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ2" t="inlineStr"/>
+      <c r="BK2" t="inlineStr"/>
+      <c r="BL2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM2" t="inlineStr"/>
+      <c r="BN2" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO2" t="inlineStr"/>
+      <c r="BP2" t="inlineStr"/>
+      <c r="BQ2" t="inlineStr"/>
+      <c r="BR2" t="inlineStr"/>
+      <c r="BS2" t="inlineStr"/>
+      <c r="BT2" t="inlineStr"/>
+      <c r="BU2" t="inlineStr"/>
+      <c r="BV2" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW2" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX2" t="inlineStr"/>
+      <c r="BY2" t="inlineStr"/>
+      <c r="BZ2" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA2" t="inlineStr"/>
+      <c r="CB2" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC2" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD2" t="inlineStr"/>
+      <c r="CE2" t="inlineStr"/>
+      <c r="CF2" t="inlineStr"/>
+      <c r="CG2" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH2" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="CI2" t="n">
+        <v>383612</v>
+      </c>
+      <c r="CJ2" t="n">
+        <v>665926</v>
+      </c>
+      <c r="CK2" t="n">
+        <v>732518</v>
+      </c>
+      <c r="CL2" t="n">
+        <v>279688</v>
+      </c>
+      <c r="CM2" t="inlineStr"/>
+      <c r="CN2" t="inlineStr"/>
+      <c r="CO2" t="inlineStr"/>
+      <c r="CP2" t="inlineStr"/>
+      <c r="CQ2" t="inlineStr"/>
+      <c r="CR2" t="inlineStr"/>
+      <c r="CS2" t="inlineStr"/>
+      <c r="CT2" t="inlineStr"/>
+      <c r="CU2" t="inlineStr"/>
+      <c r="CV2" t="inlineStr"/>
+      <c r="CW2" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX2" t="n">
+        <v>8</v>
+      </c>
+      <c r="CY2" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ2" t="inlineStr">
+        <is>
+          <t>400A</t>
+        </is>
+      </c>
+      <c r="DA2" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB2" t="inlineStr"/>
+      <c r="DC2" t="inlineStr"/>
+      <c r="DD2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>46256</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>480</v>
+      </c>
+      <c r="D3" t="n">
+        <v>4.0024</v>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" s="1" t="n">
+        <v>46257.93140291666</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>4.0024</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>201862</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0</v>
+      </c>
+      <c r="T3" t="n">
+        <v>807934</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>(휴일) 09:00~18:00</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>67,500</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
+      <c r="AR3" t="inlineStr"/>
+      <c r="AS3" t="inlineStr"/>
+      <c r="AT3" t="inlineStr"/>
+      <c r="AU3" t="inlineStr"/>
+      <c r="AV3" t="inlineStr"/>
+      <c r="AW3" t="inlineStr"/>
+      <c r="AX3" t="inlineStr"/>
+      <c r="AY3" t="inlineStr"/>
+      <c r="AZ3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG3" t="inlineStr">
+        <is>
+          <t>91주8839 (스타렉스) || 95가0175 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH3" t="inlineStr">
+        <is>
+          <t>60 || 60</t>
+        </is>
+      </c>
+      <c r="BI3" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ3" t="inlineStr">
+        <is>
+          <t>||</t>
+        </is>
+      </c>
+      <c r="BK3" t="inlineStr"/>
+      <c r="BL3" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM3" t="inlineStr"/>
+      <c r="BN3" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO3" t="inlineStr"/>
+      <c r="BP3" t="inlineStr"/>
+      <c r="BQ3" t="inlineStr"/>
+      <c r="BR3" t="inlineStr"/>
+      <c r="BS3" t="inlineStr"/>
+      <c r="BT3" t="inlineStr"/>
+      <c r="BU3" t="inlineStr"/>
+      <c r="BV3" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW3" t="inlineStr"/>
+      <c r="BX3" t="inlineStr"/>
+      <c r="BY3" t="inlineStr"/>
+      <c r="BZ3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA3" t="inlineStr"/>
+      <c r="CB3" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC3" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD3" t="inlineStr"/>
+      <c r="CE3" t="inlineStr"/>
+      <c r="CF3" t="inlineStr"/>
+      <c r="CG3" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH3" t="n">
+        <v>4.0024</v>
+      </c>
+      <c r="CI3" t="n">
+        <v>150326</v>
+      </c>
+      <c r="CJ3" t="n">
+        <v>260956</v>
+      </c>
+      <c r="CK3" t="n">
+        <v>287051</v>
+      </c>
+      <c r="CL3" t="n">
+        <v>109601</v>
+      </c>
+      <c r="CM3" t="inlineStr"/>
+      <c r="CN3" t="inlineStr"/>
+      <c r="CO3" t="inlineStr"/>
+      <c r="CP3" t="inlineStr"/>
+      <c r="CQ3" t="inlineStr"/>
+      <c r="CR3" t="inlineStr"/>
+      <c r="CS3" t="inlineStr"/>
+      <c r="CT3" t="inlineStr"/>
+      <c r="CU3" t="inlineStr"/>
+      <c r="CV3" t="inlineStr"/>
+      <c r="CW3" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX3" t="n">
+        <v>4</v>
+      </c>
+      <c r="CY3" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ3" t="inlineStr">
+        <is>
+          <t>300A</t>
+        </is>
+      </c>
+      <c r="DA3" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB3" t="inlineStr"/>
+      <c r="DC3" t="inlineStr"/>
+      <c r="DD3" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>46241</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>중앙지사</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>480</v>
+      </c>
+      <c r="D4" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="E4" t="inlineStr"/>
+      <c r="F4" s="1" t="n">
+        <v>46258.37184412037</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>부장 주진철</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>PAUT MX2(OMNI2-103085)</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>201863</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>2061744</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>PAUT</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~21:00</t>
+        </is>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>부장 박광복</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>(주간) 09:00~21:00</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>12,000</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
+      <c r="AR4" t="inlineStr"/>
+      <c r="AS4" t="inlineStr"/>
+      <c r="AT4" t="inlineStr"/>
+      <c r="AU4" t="inlineStr"/>
+      <c r="AV4" t="inlineStr"/>
+      <c r="AW4" t="inlineStr"/>
+      <c r="AX4" t="inlineStr"/>
+      <c r="AY4" t="inlineStr"/>
+      <c r="AZ4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG4" t="inlineStr">
+        <is>
+          <t>81도8458 (스타렉스)</t>
+        </is>
+      </c>
+      <c r="BH4" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="BI4" t="inlineStr">
+        <is>
+          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
+        </is>
+      </c>
+      <c r="BJ4" t="inlineStr"/>
+      <c r="BK4" t="inlineStr"/>
+      <c r="BL4" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM4" t="inlineStr"/>
+      <c r="BN4" t="inlineStr">
+        <is>
+          <t>한국지역난방공사 중앙지사</t>
+        </is>
+      </c>
+      <c r="BO4" t="inlineStr"/>
+      <c r="BP4" t="inlineStr"/>
+      <c r="BQ4" t="inlineStr"/>
+      <c r="BR4" t="inlineStr"/>
+      <c r="BS4" t="inlineStr"/>
+      <c r="BT4" t="inlineStr"/>
+      <c r="BU4" t="inlineStr"/>
+      <c r="BV4" t="inlineStr">
+        <is>
+          <t>Pipe</t>
+        </is>
+      </c>
+      <c r="BW4" t="inlineStr">
+        <is>
+          <t>KS B ISO 13588</t>
+        </is>
+      </c>
+      <c r="BX4" t="inlineStr"/>
+      <c r="BY4" t="inlineStr"/>
+      <c r="BZ4" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="CA4" t="inlineStr"/>
+      <c r="CB4" t="inlineStr">
+        <is>
+          <t>일반</t>
+        </is>
+      </c>
+      <c r="CC4" t="inlineStr">
+        <is>
+          <t>300A 이상 (1.0)</t>
+        </is>
+      </c>
+      <c r="CD4" t="inlineStr"/>
+      <c r="CE4" t="inlineStr"/>
+      <c r="CF4" t="inlineStr"/>
+      <c r="CG4" t="n">
+        <v>1</v>
+      </c>
+      <c r="CH4" t="n">
+        <v>10.2136</v>
+      </c>
+      <c r="CI4" t="n">
+        <v>383612</v>
+      </c>
+      <c r="CJ4" t="n">
+        <v>665926</v>
+      </c>
+      <c r="CK4" t="n">
+        <v>732518</v>
+      </c>
+      <c r="CL4" t="n">
+        <v>279688</v>
+      </c>
+      <c r="CM4" t="inlineStr"/>
+      <c r="CN4" t="inlineStr"/>
+      <c r="CO4" t="inlineStr"/>
+      <c r="CP4" t="inlineStr"/>
+      <c r="CQ4" t="inlineStr"/>
+      <c r="CR4" t="inlineStr"/>
+      <c r="CS4" t="inlineStr"/>
+      <c r="CT4" t="inlineStr"/>
+      <c r="CU4" t="inlineStr"/>
+      <c r="CV4" t="inlineStr"/>
+      <c r="CW4" t="inlineStr">
+        <is>
+          <t>ORI</t>
+        </is>
+      </c>
+      <c r="CX4" t="n">
+        <v>8</v>
+      </c>
+      <c r="CY4" t="n">
+        <v>0</v>
+      </c>
+      <c r="CZ4" t="inlineStr">
+        <is>
+          <t>400A</t>
+        </is>
+      </c>
+      <c r="DA4" t="inlineStr">
+        <is>
+          <t>열배관</t>
+        </is>
+      </c>
+      <c r="DB4" t="inlineStr"/>
+      <c r="DC4" t="inlineStr"/>
+      <c r="DD4" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: Add PDF Editor zoom/scroll, fix monthly report photo filter, and improve KOGAS daily log
- PDF 편집기에 화면 확대/축소 및 스크롤 기능 추가

- 월간 누적진도보고서 생성 시 타 월 사진 제외하도록 필터 복구

- KOGAS 작업일보에 자동 집계(auto_calculate_and_save) 로직 추가

- KOGAS 작업일보 관경(인치) 기준 변경 및 구간정보 텍스트박스 동적 생성 적용
</commit_message>
<xml_diff>
--- a/home/data/Material_Inventory.xlsx
+++ b/home/data/Material_Inventory.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Materials" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Budget" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Materials" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Transactions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="MonthlyUsage" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="DailyUsage" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Budget" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Settings" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -21,10 +21,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -54,9 +51,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -24725,7 +24721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DD4"/>
+  <dimension ref="A1:DC1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -25263,797 +25259,6 @@
         <is>
           <t>DailyMemo</t>
         </is>
-      </c>
-      <c r="DD1" t="inlineStr">
-        <is>
-          <t>수량</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>46242</v>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C2" t="n">
-        <v>480</v>
-      </c>
-      <c r="D2" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="F2" s="1" t="n">
-        <v>46257.92779054398</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>201863</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" t="n">
-        <v>2061744</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>(휴일) 10:00~17:00</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>52,500</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z2" t="inlineStr">
-        <is>
-          <t>(휴일) 10:00~17:00</t>
-        </is>
-      </c>
-      <c r="AA2" t="inlineStr">
-        <is>
-          <t>52,500</t>
-        </is>
-      </c>
-      <c r="AB2" t="inlineStr"/>
-      <c r="AC2" t="inlineStr"/>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
-      <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
-      <c r="AH2" t="inlineStr"/>
-      <c r="AI2" t="inlineStr"/>
-      <c r="AJ2" t="inlineStr"/>
-      <c r="AK2" t="inlineStr"/>
-      <c r="AL2" t="inlineStr"/>
-      <c r="AM2" t="inlineStr"/>
-      <c r="AN2" t="inlineStr"/>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="inlineStr"/>
-      <c r="AQ2" t="inlineStr"/>
-      <c r="AR2" t="inlineStr"/>
-      <c r="AS2" t="inlineStr"/>
-      <c r="AT2" t="inlineStr"/>
-      <c r="AU2" t="inlineStr"/>
-      <c r="AV2" t="inlineStr"/>
-      <c r="AW2" t="inlineStr"/>
-      <c r="AX2" t="inlineStr"/>
-      <c r="AY2" t="inlineStr"/>
-      <c r="AZ2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="inlineStr">
-        <is>
-          <t>81도8458 (스타렉스)</t>
-        </is>
-      </c>
-      <c r="BH2" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="BI2" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ2" t="inlineStr"/>
-      <c r="BK2" t="inlineStr"/>
-      <c r="BL2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="inlineStr">
-        <is>
-          <t>한국지역난방공사 중앙지사</t>
-        </is>
-      </c>
-      <c r="BO2" t="inlineStr"/>
-      <c r="BP2" t="inlineStr"/>
-      <c r="BQ2" t="inlineStr"/>
-      <c r="BR2" t="inlineStr"/>
-      <c r="BS2" t="inlineStr"/>
-      <c r="BT2" t="inlineStr"/>
-      <c r="BU2" t="inlineStr"/>
-      <c r="BV2" t="inlineStr">
-        <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW2" t="inlineStr">
-        <is>
-          <t>KS B ISO 13588</t>
-        </is>
-      </c>
-      <c r="BX2" t="inlineStr"/>
-      <c r="BY2" t="inlineStr"/>
-      <c r="BZ2" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA2" t="inlineStr"/>
-      <c r="CB2" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC2" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD2" t="inlineStr"/>
-      <c r="CE2" t="inlineStr"/>
-      <c r="CF2" t="inlineStr"/>
-      <c r="CG2" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH2" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="CI2" t="n">
-        <v>383612</v>
-      </c>
-      <c r="CJ2" t="n">
-        <v>665926</v>
-      </c>
-      <c r="CK2" t="n">
-        <v>732518</v>
-      </c>
-      <c r="CL2" t="n">
-        <v>279688</v>
-      </c>
-      <c r="CM2" t="inlineStr"/>
-      <c r="CN2" t="inlineStr"/>
-      <c r="CO2" t="inlineStr"/>
-      <c r="CP2" t="inlineStr"/>
-      <c r="CQ2" t="inlineStr"/>
-      <c r="CR2" t="inlineStr"/>
-      <c r="CS2" t="inlineStr"/>
-      <c r="CT2" t="inlineStr"/>
-      <c r="CU2" t="inlineStr"/>
-      <c r="CV2" t="inlineStr"/>
-      <c r="CW2" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX2" t="n">
-        <v>8</v>
-      </c>
-      <c r="CY2" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ2" t="inlineStr">
-        <is>
-          <t>400A</t>
-        </is>
-      </c>
-      <c r="DA2" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB2" t="inlineStr"/>
-      <c r="DC2" t="inlineStr"/>
-      <c r="DD2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>46256</v>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C3" t="n">
-        <v>480</v>
-      </c>
-      <c r="D3" t="n">
-        <v>4.0024</v>
-      </c>
-      <c r="E3" t="inlineStr"/>
-      <c r="F3" s="1" t="n">
-        <v>46257.93140291666</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>4.0024</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>201862</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0</v>
-      </c>
-      <c r="T3" t="n">
-        <v>807934</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>0</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>67,500</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z3" t="inlineStr">
-        <is>
-          <t>(휴일) 09:00~18:00</t>
-        </is>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>67,500</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr"/>
-      <c r="AC3" t="inlineStr"/>
-      <c r="AD3" t="inlineStr"/>
-      <c r="AE3" t="inlineStr"/>
-      <c r="AF3" t="inlineStr"/>
-      <c r="AG3" t="inlineStr"/>
-      <c r="AH3" t="inlineStr"/>
-      <c r="AI3" t="inlineStr"/>
-      <c r="AJ3" t="inlineStr"/>
-      <c r="AK3" t="inlineStr"/>
-      <c r="AL3" t="inlineStr"/>
-      <c r="AM3" t="inlineStr"/>
-      <c r="AN3" t="inlineStr"/>
-      <c r="AO3" t="inlineStr"/>
-      <c r="AP3" t="inlineStr"/>
-      <c r="AQ3" t="inlineStr"/>
-      <c r="AR3" t="inlineStr"/>
-      <c r="AS3" t="inlineStr"/>
-      <c r="AT3" t="inlineStr"/>
-      <c r="AU3" t="inlineStr"/>
-      <c r="AV3" t="inlineStr"/>
-      <c r="AW3" t="inlineStr"/>
-      <c r="AX3" t="inlineStr"/>
-      <c r="AY3" t="inlineStr"/>
-      <c r="AZ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG3" t="inlineStr">
-        <is>
-          <t>91주8839 (스타렉스) || 95가0175 (스타렉스)</t>
-        </is>
-      </c>
-      <c r="BH3" t="inlineStr">
-        <is>
-          <t>60 || 60</t>
-        </is>
-      </c>
-      <c r="BI3" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함 || out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ3" t="inlineStr">
-        <is>
-          <t>||</t>
-        </is>
-      </c>
-      <c r="BK3" t="inlineStr"/>
-      <c r="BL3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM3" t="inlineStr"/>
-      <c r="BN3" t="inlineStr">
-        <is>
-          <t>한국지역난방공사 중앙지사</t>
-        </is>
-      </c>
-      <c r="BO3" t="inlineStr"/>
-      <c r="BP3" t="inlineStr"/>
-      <c r="BQ3" t="inlineStr"/>
-      <c r="BR3" t="inlineStr"/>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="inlineStr"/>
-      <c r="BU3" t="inlineStr"/>
-      <c r="BV3" t="inlineStr">
-        <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW3" t="inlineStr"/>
-      <c r="BX3" t="inlineStr"/>
-      <c r="BY3" t="inlineStr"/>
-      <c r="BZ3" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA3" t="inlineStr"/>
-      <c r="CB3" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC3" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD3" t="inlineStr"/>
-      <c r="CE3" t="inlineStr"/>
-      <c r="CF3" t="inlineStr"/>
-      <c r="CG3" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH3" t="n">
-        <v>4.0024</v>
-      </c>
-      <c r="CI3" t="n">
-        <v>150326</v>
-      </c>
-      <c r="CJ3" t="n">
-        <v>260956</v>
-      </c>
-      <c r="CK3" t="n">
-        <v>287051</v>
-      </c>
-      <c r="CL3" t="n">
-        <v>109601</v>
-      </c>
-      <c r="CM3" t="inlineStr"/>
-      <c r="CN3" t="inlineStr"/>
-      <c r="CO3" t="inlineStr"/>
-      <c r="CP3" t="inlineStr"/>
-      <c r="CQ3" t="inlineStr"/>
-      <c r="CR3" t="inlineStr"/>
-      <c r="CS3" t="inlineStr"/>
-      <c r="CT3" t="inlineStr"/>
-      <c r="CU3" t="inlineStr"/>
-      <c r="CV3" t="inlineStr"/>
-      <c r="CW3" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX3" t="n">
-        <v>4</v>
-      </c>
-      <c r="CY3" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ3" t="inlineStr">
-        <is>
-          <t>300A</t>
-        </is>
-      </c>
-      <c r="DA3" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB3" t="inlineStr"/>
-      <c r="DC3" t="inlineStr"/>
-      <c r="DD3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>46241</v>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>중앙지사</t>
-        </is>
-      </c>
-      <c r="C4" t="n">
-        <v>480</v>
-      </c>
-      <c r="D4" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" s="1" t="n">
-        <v>46258.37184412037</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0</v>
-      </c>
-      <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>부장 주진철</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>PAUT MX2(OMNI2-103085)</t>
-        </is>
-      </c>
-      <c r="P4" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="Q4" t="n">
-        <v>201863</v>
-      </c>
-      <c r="R4" t="n">
-        <v>0</v>
-      </c>
-      <c r="S4" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" t="n">
-        <v>2061744</v>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>PAUT</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>0</v>
-      </c>
-      <c r="W4" t="inlineStr">
-        <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="X4" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="Y4" t="inlineStr">
-        <is>
-          <t>부장 박광복</t>
-        </is>
-      </c>
-      <c r="Z4" t="inlineStr">
-        <is>
-          <t>(주간) 09:00~21:00</t>
-        </is>
-      </c>
-      <c r="AA4" t="inlineStr">
-        <is>
-          <t>12,000</t>
-        </is>
-      </c>
-      <c r="AB4" t="inlineStr"/>
-      <c r="AC4" t="inlineStr"/>
-      <c r="AD4" t="inlineStr"/>
-      <c r="AE4" t="inlineStr"/>
-      <c r="AF4" t="inlineStr"/>
-      <c r="AG4" t="inlineStr"/>
-      <c r="AH4" t="inlineStr"/>
-      <c r="AI4" t="inlineStr"/>
-      <c r="AJ4" t="inlineStr"/>
-      <c r="AK4" t="inlineStr"/>
-      <c r="AL4" t="inlineStr"/>
-      <c r="AM4" t="inlineStr"/>
-      <c r="AN4" t="inlineStr"/>
-      <c r="AO4" t="inlineStr"/>
-      <c r="AP4" t="inlineStr"/>
-      <c r="AQ4" t="inlineStr"/>
-      <c r="AR4" t="inlineStr"/>
-      <c r="AS4" t="inlineStr"/>
-      <c r="AT4" t="inlineStr"/>
-      <c r="AU4" t="inlineStr"/>
-      <c r="AV4" t="inlineStr"/>
-      <c r="AW4" t="inlineStr"/>
-      <c r="AX4" t="inlineStr"/>
-      <c r="AY4" t="inlineStr"/>
-      <c r="AZ4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG4" t="inlineStr">
-        <is>
-          <t>81도8458 (스타렉스)</t>
-        </is>
-      </c>
-      <c r="BH4" t="inlineStr">
-        <is>
-          <t>60</t>
-        </is>
-      </c>
-      <c r="BI4" t="inlineStr">
-        <is>
-          <t>out_exterior:양호|out_cleanliness:양호|out_cleaning:함|out_locking:안함|in_exterior:양호|in_cleanliness:양호|in_cleaning:함|in_locking:안함</t>
-        </is>
-      </c>
-      <c r="BJ4" t="inlineStr"/>
-      <c r="BK4" t="inlineStr"/>
-      <c r="BL4" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM4" t="inlineStr"/>
-      <c r="BN4" t="inlineStr">
-        <is>
-          <t>한국지역난방공사 중앙지사</t>
-        </is>
-      </c>
-      <c r="BO4" t="inlineStr"/>
-      <c r="BP4" t="inlineStr"/>
-      <c r="BQ4" t="inlineStr"/>
-      <c r="BR4" t="inlineStr"/>
-      <c r="BS4" t="inlineStr"/>
-      <c r="BT4" t="inlineStr"/>
-      <c r="BU4" t="inlineStr"/>
-      <c r="BV4" t="inlineStr">
-        <is>
-          <t>Pipe</t>
-        </is>
-      </c>
-      <c r="BW4" t="inlineStr">
-        <is>
-          <t>KS B ISO 13588</t>
-        </is>
-      </c>
-      <c r="BX4" t="inlineStr"/>
-      <c r="BY4" t="inlineStr"/>
-      <c r="BZ4" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-      <c r="CA4" t="inlineStr"/>
-      <c r="CB4" t="inlineStr">
-        <is>
-          <t>일반</t>
-        </is>
-      </c>
-      <c r="CC4" t="inlineStr">
-        <is>
-          <t>300A 이상 (1.0)</t>
-        </is>
-      </c>
-      <c r="CD4" t="inlineStr"/>
-      <c r="CE4" t="inlineStr"/>
-      <c r="CF4" t="inlineStr"/>
-      <c r="CG4" t="n">
-        <v>1</v>
-      </c>
-      <c r="CH4" t="n">
-        <v>10.2136</v>
-      </c>
-      <c r="CI4" t="n">
-        <v>383612</v>
-      </c>
-      <c r="CJ4" t="n">
-        <v>665926</v>
-      </c>
-      <c r="CK4" t="n">
-        <v>732518</v>
-      </c>
-      <c r="CL4" t="n">
-        <v>279688</v>
-      </c>
-      <c r="CM4" t="inlineStr"/>
-      <c r="CN4" t="inlineStr"/>
-      <c r="CO4" t="inlineStr"/>
-      <c r="CP4" t="inlineStr"/>
-      <c r="CQ4" t="inlineStr"/>
-      <c r="CR4" t="inlineStr"/>
-      <c r="CS4" t="inlineStr"/>
-      <c r="CT4" t="inlineStr"/>
-      <c r="CU4" t="inlineStr"/>
-      <c r="CV4" t="inlineStr"/>
-      <c r="CW4" t="inlineStr">
-        <is>
-          <t>ORI</t>
-        </is>
-      </c>
-      <c r="CX4" t="n">
-        <v>8</v>
-      </c>
-      <c r="CY4" t="n">
-        <v>0</v>
-      </c>
-      <c r="CZ4" t="inlineStr">
-        <is>
-          <t>400A</t>
-        </is>
-      </c>
-      <c r="DA4" t="inlineStr">
-        <is>
-          <t>열배관</t>
-        </is>
-      </c>
-      <c r="DB4" t="inlineStr"/>
-      <c r="DC4" t="inlineStr"/>
-      <c r="DD4" t="n">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>